<commit_message>
Daily EOD data and reports for 2026-08-07
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260807.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260807.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.5</v>
+        <v>1.502</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.035</v>
+        <v>0.037</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.39%</t>
+          <t>2.53%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>229771.5</v>
+        <v>230077.86</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>5361.33</v>
+        <v>5667.7</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.385</v>
+        <v>2.41</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.075</v>
+        <v>0.1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3.25%</t>
+          <t>4.33%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>166950</v>
+        <v>168700</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>5250</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="6">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>62.84</v>
+        <v>62.87</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.02</v>
+        <v>0.05</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.03%</t>
+          <t>0.08%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>695324.6</v>
+        <v>695656.55</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>221.3</v>
+        <v>553.25</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>177.66</v>
+        <v>177.31</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-2.21</v>
+        <v>-2.56</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-1.23%</t>
+          <t>-1.42%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>131.62</v>
+        <v>131.91</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-0.74</v>
+        <v>-0.45</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.56%</t>
+          <t>-0.34%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>526480</v>
+        <v>527640</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-2960</v>
+        <v>-1800</v>
       </c>
     </row>
     <row r="12">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>37.93</v>
+        <v>37.94</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.6</v>
+        <v>-0.59</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-1.56%</t>
+          <t>-1.53%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1733758.06</v>
+        <v>1737306.37</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>5832.03</v>
+        <v>9380.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>